<commit_message>
GateX: plain-language dashboard, charted PDF report, new checks, updated docs
</commit_message>
<xml_diff>
--- a/samples/talentra/talentra-schema-d2.xlsx
+++ b/samples/talentra/talentra-schema-d2.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="192">
   <si>
     <t>How to fill in this scorecard</t>
   </si>
@@ -34,10 +34,13 @@
     <t xml:space="preserve">  id, version, judges are required. "judges" must start with D1 (a schema design) or D3 (an output document).</t>
   </si>
   <si>
-    <t xml:space="preserve">  frozen must be yes. A scorecard that is not frozen is refused, so the target cannot move mid-evaluation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  accept and refine are the green and amber thresholds (default 90 and 75). approval says who approved it; if it says "pending" or "draft", every report is marked provisional.</t>
+    <t xml:space="preserve">  frozen is optional: the app freezes every scorecard by its hash when work is submitted, so the target cannot move mid-evaluation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  accept and refine are the green and amber thresholds (default 90 and 75). approval (optional) is shown in the report header as where the scorecard came from.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  unmeasured (optional) = skip (default: a question the file holds nothing for is left out of the score) or zero (it counts as 0).</t>
   </si>
   <si>
     <t xml:space="preserve">  Format the version cell as Text, or Excel turns 1.0 into 1.</t>
@@ -61,7 +64,10 @@
     <t xml:space="preserve">  Weight = importance (any positive number; they need not add to 100). Critical = yes means it must score 4 or more or the verdict cannot be green.</t>
   </si>
   <si>
-    <t xml:space="preserve">  Measured by = code (counted exactly), raters (the AI examiners score 0-5 against your anchors) or human (only a person can supply it).</t>
+    <t xml:space="preserve">  Measured by = code (counted exactly) or raters (the AI examiners score 0-5 against your anchors). Nothing waits for a person:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        human is still accepted, and such a row is scored by the examiners from what the file shows (standard anchors if none are given).</t>
   </si>
   <si>
     <t xml:space="preserve">  raters: fill all six Anchor columns, saying what a 0, 1, 2, 3, 4 and 5 mean.</t>
@@ -79,9 +85,6 @@
     <t xml:space="preserve">        strict = 1:5, 0.97:4, 0.9:3, 0.75:2, 0.01:1     exact = 1:5, 0.01:1 (one mistake fails it)</t>
   </si>
   <si>
-    <t xml:space="preserve">  human: fill Needs, saying what the person must provide (for example a scored author interview).</t>
-  </si>
-  <si>
     <t xml:space="preserve">  Fix = what to do when a code check fails. Return to = which stage the author goes back to (Discover, Define, Generate, Analyse, Validate, Refine).</t>
   </si>
   <si>
@@ -133,7 +136,7 @@
     <t>approval</t>
   </si>
   <si>
-    <t>Draft by the assistant, pending mentor approval</t>
+    <t>Sample scorecard for the Talentra workbook, used as it is</t>
   </si>
   <si>
     <t>accept</t>
@@ -241,6 +244,9 @@
     <t>Return to</t>
   </si>
   <si>
+    <t>Reads</t>
+  </si>
+  <si>
     <t>C01</t>
   </si>
   <si>
@@ -562,7 +568,25 @@
     <t>Author understanding</t>
   </si>
   <si>
-    <t>human</t>
+    <t>A scored author interview (0-5) run by the mentor. No edit to the document can prove the author understands it. Score only what the file itself shows for this. If the file holds no evidence for it at all, mark it not measurable.</t>
+  </si>
+  <si>
+    <t>Every item meets it, with nothing missing.</t>
+  </si>
+  <si>
+    <t>Nearly all items meet it, with one minor gap.</t>
+  </si>
+  <si>
+    <t>Most items meet it, with clear gaps left.</t>
+  </si>
+  <si>
+    <t>About half of the items meet it, or there are serious gaps.</t>
+  </si>
+  <si>
+    <t>A few items meet it; most do not.</t>
+  </si>
+  <si>
+    <t>None of what the question asks for is in the file.</t>
   </si>
   <si>
     <t>A scored author interview (0-5) run by the mentor. No edit to the document can prove the author understands it.</t>
@@ -965,7 +989,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="150" customWidth="1"/>
@@ -1023,16 +1047,16 @@
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1048,16 +1072,16 @@
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1103,12 +1127,17 @@
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>1</v>
+        <v>23</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>23</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -1128,71 +1157,71 @@
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B9">
         <v>90</v>
@@ -1200,7 +1229,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B10">
         <v>75</v>
@@ -1225,72 +1254,72 @@
   <sheetData>
     <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3" t="s">
         <v>49</v>
-      </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3" t="s">
-        <v>50</v>
-      </c>
-      <c r="D3" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B4">
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B5">
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="4:4" x14ac:dyDescent="0.25"/>
@@ -1505,7 +1534,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S201"/>
+  <dimension ref="A1:T201"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1518,85 +1547,89 @@
     <col min="16" max="16" width="26" customWidth="1"/>
     <col min="17" max="18" width="40" customWidth="1"/>
     <col min="19" max="19" width="12" customWidth="1"/>
+    <col min="20" max="20" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+      <c r="T1" s="4" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C2" s="5">
         <v>5</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G2" s="5" t="s">
         <v>1</v>
@@ -1620,16 +1653,16 @@
         <v>1</v>
       </c>
       <c r="N2" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="O2" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="P2" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="Q2" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="R2" s="5" t="s">
         <v>1</v>
@@ -1637,25 +1670,28 @@
       <c r="S2" s="5" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T2" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C3" s="5">
         <v>8</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>1</v>
@@ -1679,16 +1715,16 @@
         <v>1</v>
       </c>
       <c r="N3" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="R3" s="5" t="s">
         <v>1</v>
@@ -1696,13 +1732,16 @@
       <c r="S3" s="5" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T3" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C4" s="5">
         <v>4</v>
@@ -1711,7 +1750,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>1</v>
@@ -1738,16 +1777,16 @@
         <v>1</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="R4" s="5" t="s">
         <v>1</v>
@@ -1755,13 +1794,16 @@
       <c r="S4" s="5" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T4" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C5" s="5">
         <v>4</v>
@@ -1770,7 +1812,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>1</v>
@@ -1797,16 +1839,16 @@
         <v>1</v>
       </c>
       <c r="N5" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="O5" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="P5" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="Q5" s="5" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="R5" s="5" t="s">
         <v>1</v>
@@ -1814,22 +1856,25 @@
       <c r="S5" s="5" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T5" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C6" s="5">
         <v>6</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>1</v>
@@ -1856,16 +1901,16 @@
         <v>1</v>
       </c>
       <c r="N6" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="R6" s="5" t="s">
         <v>1</v>
@@ -1873,25 +1918,28 @@
       <c r="S6" s="5" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T6" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C7" s="5">
         <v>5</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="G7" s="5" t="s">
         <v>1</v>
@@ -1915,16 +1963,16 @@
         <v>1</v>
       </c>
       <c r="N7" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="O7" s="5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="P7" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="Q7" s="5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="R7" s="5" t="s">
         <v>1</v>
@@ -1932,13 +1980,16 @@
       <c r="S7" s="5" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T7" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C8" s="5">
         <v>3</v>
@@ -1947,7 +1998,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F8" s="5" t="s">
         <v>1</v>
@@ -1974,16 +2025,16 @@
         <v>1</v>
       </c>
       <c r="N8" s="5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="O8" s="5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="P8" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="Q8" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="R8" s="5" t="s">
         <v>1</v>
@@ -1991,13 +2042,16 @@
       <c r="S8" s="5" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T8" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C9" s="5">
         <v>4</v>
@@ -2006,10 +2060,10 @@
         <v>1</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>1</v>
@@ -2033,16 +2087,16 @@
         <v>1</v>
       </c>
       <c r="N9" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="O9" s="5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="P9" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="Q9" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="R9" s="5" t="s">
         <v>1</v>
@@ -2050,13 +2104,16 @@
       <c r="S9" s="5" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T9" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C10" s="5">
         <v>3</v>
@@ -2065,10 +2122,10 @@
         <v>1</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>1</v>
@@ -2092,16 +2149,16 @@
         <v>1</v>
       </c>
       <c r="N10" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="O10" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="P10" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="Q10" s="5" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="R10" s="5" t="s">
         <v>1</v>
@@ -2109,13 +2166,16 @@
       <c r="S10" s="5" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T10" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C11" s="5">
         <v>10</v>
@@ -2124,31 +2184,31 @@
         <v>1</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>1</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="L11" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="M11" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="N11" s="5" t="s">
         <v>1</v>
@@ -2168,13 +2228,16 @@
       <c r="S11" s="5" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T11" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C12" s="5">
         <v>8</v>
@@ -2183,31 +2246,31 @@
         <v>1</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G12" s="5" t="s">
         <v>1</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="L12" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="M12" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="N12" s="5" t="s">
         <v>1</v>
@@ -2227,13 +2290,16 @@
       <c r="S12" s="5" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T12" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C13" s="5">
         <v>6</v>
@@ -2242,31 +2308,31 @@
         <v>1</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G13" s="5" t="s">
         <v>1</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="L13" s="5" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="M13" s="5" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="N13" s="5" t="s">
         <v>1</v>
@@ -2286,46 +2352,49 @@
       <c r="S13" s="5" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T13" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C14" s="5">
         <v>12</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="G14" s="5" t="s">
         <v>1</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="L14" s="5" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="M14" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="N14" s="5" t="s">
         <v>1</v>
@@ -2343,15 +2412,18 @@
         <v>1</v>
       </c>
       <c r="S14" s="5" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+        <v>163</v>
+      </c>
+      <c r="T14" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C15" s="5">
         <v>6</v>
@@ -2360,31 +2432,31 @@
         <v>1</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="G15" s="5" t="s">
         <v>1</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="L15" s="5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="M15" s="5" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="N15" s="5" t="s">
         <v>1</v>
@@ -2404,13 +2476,16 @@
       <c r="S15" s="5" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T15" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C16" s="5">
         <v>6</v>
@@ -2419,31 +2494,31 @@
         <v>1</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="G16" s="5" t="s">
         <v>1</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="L16" s="5" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="N16" s="5" t="s">
         <v>1</v>
@@ -2463,46 +2538,49 @@
       <c r="S16" s="5" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T16" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C17" s="5">
         <v>10</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>182</v>
+        <v>128</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>1</v>
+        <v>184</v>
       </c>
       <c r="G17" s="5" t="s">
         <v>1</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>1</v>
+        <v>185</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>1</v>
+        <v>186</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>1</v>
+        <v>187</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>1</v>
+        <v>188</v>
       </c>
       <c r="L17" s="5" t="s">
-        <v>1</v>
+        <v>189</v>
       </c>
       <c r="M17" s="5" t="s">
-        <v>1</v>
+        <v>190</v>
       </c>
       <c r="N17" s="5" t="s">
         <v>1</v>
@@ -2517,9 +2595,12 @@
         <v>1</v>
       </c>
       <c r="R17" s="5" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="S17" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="T17" s="5" t="s">
         <v>1</v>
       </c>
     </row>

</xml_diff>